<commit_message>
Fix invisible verdict text (explicit black font)
</commit_message>
<xml_diff>
--- a/data/human_calibration/human_calibration_labeling.xlsx
+++ b/data/human_calibration/human_calibration_labeling.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,21 +29,31 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="FF000000"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
+      <color rgb="FF000000"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="4">
@@ -78,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -96,6 +106,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -703,7 +714,7 @@
           <t>-0.15090543259557343</t>
         </is>
       </c>
-      <c r="F2" s="6" t="n"/>
+      <c r="F2" s="9" t="n"/>
     </row>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="5" t="n">
@@ -729,7 +740,7 @@
           <t>3291438.0</t>
         </is>
       </c>
-      <c r="F3" s="6" t="n"/>
+      <c r="F3" s="9" t="n"/>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="5" t="n">
@@ -755,7 +766,7 @@
           <t>2.0</t>
         </is>
       </c>
-      <c r="F4" s="6" t="n"/>
+      <c r="F4" s="9" t="n"/>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="5" t="n">
@@ -781,7 +792,7 @@
           <t>3472.0</t>
         </is>
       </c>
-      <c r="F5" s="6" t="n"/>
+      <c r="F5" s="9" t="n"/>
     </row>
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="5" t="n">
@@ -807,7 +818,7 @@
           <t>-0.1752147766323024</t>
         </is>
       </c>
-      <c r="F6" s="6" t="n"/>
+      <c r="F6" s="9" t="n"/>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="5" t="n">
@@ -833,7 +844,7 @@
           <t>0.07760000000000006</t>
         </is>
       </c>
-      <c r="F7" s="6" t="n"/>
+      <c r="F7" s="9" t="n"/>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="5" t="n">
@@ -859,7 +870,7 @@
           <t>180.0</t>
         </is>
       </c>
-      <c r="F8" s="6" t="n"/>
+      <c r="F8" s="9" t="n"/>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="5" t="n">
@@ -885,7 +896,7 @@
           <t>-2022.0</t>
         </is>
       </c>
-      <c r="F9" s="6" t="n"/>
+      <c r="F9" s="9" t="n"/>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="5" t="n">
@@ -911,7 +922,7 @@
           <t>0.7681159420289854</t>
         </is>
       </c>
-      <c r="F10" s="6" t="n"/>
+      <c r="F10" s="9" t="n"/>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="5" t="n">
@@ -937,7 +948,7 @@
           <t>13225.7556</t>
         </is>
       </c>
-      <c r="F11" s="6" t="n"/>
+      <c r="F11" s="9" t="n"/>
     </row>
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="5" t="n">
@@ -963,7 +974,7 @@
           <t>549.0</t>
         </is>
       </c>
-      <c r="F12" s="6" t="n"/>
+      <c r="F12" s="9" t="n"/>
     </row>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="5" t="n">
@@ -989,7 +1000,7 @@
           <t>5700.0</t>
         </is>
       </c>
-      <c r="F13" s="6" t="n"/>
+      <c r="F13" s="9" t="n"/>
     </row>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="5" t="n">
@@ -1015,7 +1026,7 @@
           <t>28.999999999999996</t>
         </is>
       </c>
-      <c r="F14" s="6" t="n"/>
+      <c r="F14" s="9" t="n"/>
     </row>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="5" t="n">
@@ -1041,7 +1052,7 @@
           <t>-49.0</t>
         </is>
       </c>
-      <c r="F15" s="6" t="n"/>
+      <c r="F15" s="9" t="n"/>
     </row>
     <row r="16" ht="45" customHeight="1">
       <c r="A16" s="5" t="n">
@@ -1067,7 +1078,7 @@
           <t>570400.0</t>
         </is>
       </c>
-      <c r="F16" s="6" t="n"/>
+      <c r="F16" s="9" t="n"/>
     </row>
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="5" t="n">
@@ -1093,7 +1104,7 @@
           <t>15381.0</t>
         </is>
       </c>
-      <c r="F17" s="6" t="n"/>
+      <c r="F17" s="9" t="n"/>
     </row>
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="5" t="n">
@@ -1119,7 +1130,7 @@
           <t>23.0</t>
         </is>
       </c>
-      <c r="F18" s="6" t="n"/>
+      <c r="F18" s="9" t="n"/>
     </row>
     <row r="19" ht="45" customHeight="1">
       <c r="A19" s="5" t="n">
@@ -1145,7 +1156,7 @@
           <t>119655.67</t>
         </is>
       </c>
-      <c r="F19" s="6" t="n"/>
+      <c r="F19" s="9" t="n"/>
     </row>
     <row r="20" ht="45" customHeight="1">
       <c r="A20" s="5" t="n">
@@ -1171,7 +1182,7 @@
           <t>18671.0</t>
         </is>
       </c>
-      <c r="F20" s="6" t="n"/>
+      <c r="F20" s="9" t="n"/>
     </row>
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="5" t="n">
@@ -1197,7 +1208,7 @@
           <t>0.2938388625592417</t>
         </is>
       </c>
-      <c r="F21" s="6" t="n"/>
+      <c r="F21" s="9" t="n"/>
     </row>
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="5" t="n">
@@ -1223,7 +1234,7 @@
           <t>0.8558373516456715</t>
         </is>
       </c>
-      <c r="F22" s="6" t="n"/>
+      <c r="F22" s="9" t="n"/>
     </row>
     <row r="23" ht="45" customHeight="1">
       <c r="A23" s="5" t="n">
@@ -1249,7 +1260,7 @@
           <t>0.25</t>
         </is>
       </c>
-      <c r="F23" s="6" t="n"/>
+      <c r="F23" s="9" t="n"/>
     </row>
     <row r="24" ht="45" customHeight="1">
       <c r="A24" s="5" t="n">
@@ -1275,7 +1286,7 @@
           <t>-15.8</t>
         </is>
       </c>
-      <c r="F24" s="6" t="n"/>
+      <c r="F24" s="9" t="n"/>
     </row>
     <row r="25" ht="45" customHeight="1">
       <c r="A25" s="5" t="n">
@@ -1301,7 +1312,7 @@
           <t>196941.0</t>
         </is>
       </c>
-      <c r="F25" s="6" t="n"/>
+      <c r="F25" s="9" t="n"/>
     </row>
     <row r="26" ht="45" customHeight="1">
       <c r="A26" s="5" t="n">
@@ -1327,7 +1338,7 @@
           <t>0.4</t>
         </is>
       </c>
-      <c r="F26" s="6" t="n"/>
+      <c r="F26" s="9" t="n"/>
     </row>
     <row r="27" ht="45" customHeight="1">
       <c r="A27" s="5" t="n">
@@ -1353,7 +1364,7 @@
           <t>756.0</t>
         </is>
       </c>
-      <c r="F27" s="6" t="n"/>
+      <c r="F27" s="9" t="n"/>
     </row>
     <row r="28" ht="45" customHeight="1">
       <c r="A28" s="5" t="n">
@@ -1379,7 +1390,7 @@
           <t>324.5</t>
         </is>
       </c>
-      <c r="F28" s="6" t="n"/>
+      <c r="F28" s="9" t="n"/>
     </row>
     <row r="29" ht="45" customHeight="1">
       <c r="A29" s="5" t="n">
@@ -1405,7 +1416,7 @@
           <t>2074.0</t>
         </is>
       </c>
-      <c r="F29" s="6" t="n"/>
+      <c r="F29" s="9" t="n"/>
     </row>
     <row r="30" ht="45" customHeight="1">
       <c r="A30" s="5" t="n">
@@ -1431,7 +1442,7 @@
           <t>0.32701421800947866</t>
         </is>
       </c>
-      <c r="F30" s="6" t="n"/>
+      <c r="F30" s="9" t="n"/>
     </row>
     <row r="31" ht="45" customHeight="1">
       <c r="A31" s="5" t="n">
@@ -1457,7 +1468,7 @@
           <t>60.0</t>
         </is>
       </c>
-      <c r="F31" s="6" t="n"/>
+      <c r="F31" s="9" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Remove yellow fill, add plain CSV fallback
</commit_message>
<xml_diff>
--- a/data/human_calibration/human_calibration_labeling.xlsx
+++ b/data/human_calibration/human_calibration_labeling.xlsx
@@ -56,7 +56,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -69,20 +69,28 @@
         <bgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -101,12 +109,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -501,7 +509,7 @@
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Что делать: на листе 'Разметка' — 30 вопросов, выбранных случайно (фиксированный seed) из прогона results/error_analysis_250, пропорционально распределению по источникам (TAT-DQA / FinQA / ConvFinQA). Для каждой строки в столбце F (жёлтая заливка) укажите CORRECT, если 'Ответ модели' по существу совпадает с 'Эталонным ответом', или INCORRECT — если нет.</t>
+          <t>Что делать: на листе 'Разметка' — 30 вопросов, выбранных случайно (фиксированный seed) из прогона results/error_analysis_250, пропорционально распределению по источникам (TAT-DQA / FinQA / ConvFinQA). Для каждой строки в столбце F (с рамкой) укажите CORRECT, если 'Ответ модели' по существу совпадает с 'Эталонным ответом', или INCORRECT — если нет.</t>
         </is>
       </c>
     </row>

</xml_diff>